<commit_message>
Simulated Custom vs. Normal
</commit_message>
<xml_diff>
--- a/src/main/resources/analytics/results/FinalResultsOfStrategyVsRules.xlsx
+++ b/src/main/resources/analytics/results/FinalResultsOfStrategyVsRules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Coding\BlackjackSimulator\src\main\resources\analytics\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D11B7410-DCA5-465F-82BB-A7C836FFD206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F71455-A7AE-4C2C-83AC-681F66C81277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="7710" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4908" yWindow="2316" windowWidth="21600" windowHeight="11832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,8 @@
     <externalReference r:id="rId6"/>
     <externalReference r:id="rId7"/>
     <externalReference r:id="rId8"/>
+    <externalReference r:id="rId9"/>
+    <externalReference r:id="rId10"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -262,20 +264,20 @@
       <sheetData sheetId="0">
         <row r="11">
           <cell r="B11">
-            <v>3.2476227506068453E-3</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
+            <v>-2.5169005874125664E-3</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -304,26 +306,70 @@
       <sheetData sheetId="0">
         <row r="11">
           <cell r="B11">
-            <v>-2.5169005874125664E-3</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
+            <v>3.2476227506068453E-3</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
 </file>
 
 <file path=xl/externalLinks/externalLink7.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Results"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="6">
+          <cell r="Q6">
+            <v>-1.6676403792794905E-2</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink8.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Results"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="6">
+          <cell r="Q6">
+            <v>-7.1820273972602738E-3</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink9.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
@@ -350,16 +396,16 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -689,11 +735,11 @@
         <v>6</v>
       </c>
       <c r="C5" s="1">
+        <f>[5]Results!$B$11</f>
+        <v>-2.5169005874125664E-3</v>
+      </c>
+      <c r="D5" s="1">
         <f>[6]Results!$B$11</f>
-        <v>-2.5169005874125664E-3</v>
-      </c>
-      <c r="D5" s="1">
-        <f>[5]Results!$B$11</f>
         <v>3.2476227506068453E-3</v>
       </c>
     </row>
@@ -702,16 +748,22 @@
       <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
+      <c r="C6" s="1">
+        <f>[7]Results!$Q$6</f>
+        <v>-1.6676403792794905E-2</v>
+      </c>
+      <c r="D6" s="1">
+        <f>[8]Results!$Q$6</f>
+        <v>-7.1820273972602738E-3</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D7">
-        <f ca="1">[7]Results!$B$11</f>
+      <c r="D7" s="1">
+        <f>[9]Results!$B$11</f>
         <v>-7.4210901656173349E-3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Simulated Custom >2TC vs. Normal
</commit_message>
<xml_diff>
--- a/src/main/resources/analytics/results/FinalResultsOfStrategyVsRules.xlsx
+++ b/src/main/resources/analytics/results/FinalResultsOfStrategyVsRules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Coding\BlackjackSimulator\src\main\resources\analytics\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F71455-A7AE-4C2C-83AC-681F66C81277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4ECD033-6213-4732-9350-9A3B804A517B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4908" yWindow="2316" windowWidth="21600" windowHeight="11832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4920" yWindow="3684" windowWidth="21600" windowHeight="11832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <externalReference r:id="rId8"/>
     <externalReference r:id="rId9"/>
     <externalReference r:id="rId10"/>
+    <externalReference r:id="rId11"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -170,6 +171,65 @@
           </cell>
         </row>
       </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink10.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Results"/>
+      <sheetName val="Results1"/>
+      <sheetName val="Results2"/>
+      <sheetName val="Results3"/>
+      <sheetName val="Results4"/>
+      <sheetName val="Results5"/>
+      <sheetName val="Results6"/>
+      <sheetName val="Results7"/>
+      <sheetName val="Results8"/>
+      <sheetName val="Results9"/>
+      <sheetName val="Results10"/>
+      <sheetName val="Results1 (2)"/>
+      <sheetName val="Results2 (2)"/>
+      <sheetName val="Results3 (2)"/>
+      <sheetName val="Results4 (2)"/>
+      <sheetName val="Results5 (2)"/>
+      <sheetName val="Results6 (2)"/>
+      <sheetName val="Results7 (2)"/>
+      <sheetName val="Results8 (2)"/>
+      <sheetName val="Results9 (2)"/>
+      <sheetName val="Results10 (2)"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="11">
+          <cell r="B11">
+            <v>-1.0033829565285212E-2</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -739,7 +799,7 @@
         <v>-2.5169005874125664E-3</v>
       </c>
       <c r="D5" s="1">
-        <f>[6]Results!$B$11</f>
+        <f ca="1">[6]Results!$B$11</f>
         <v>3.2476227506068453E-3</v>
       </c>
     </row>
@@ -761,6 +821,10 @@
       <c r="A7" s="4"/>
       <c r="B7" s="2" t="s">
         <v>7</v>
+      </c>
+      <c r="C7" s="1">
+        <f>[10]Results!$B$11</f>
+        <v>-1.0033829565285212E-2</v>
       </c>
       <c r="D7" s="1">
         <f>[9]Results!$B$11</f>

</xml_diff>